<commit_message>
Add reviewer-facing clarity, CIs to calibration report, and repo transparency fixes
- Add PLAIN_SUMMARY.md: plain-language entry point for surgeon collaborators
- README: narrative-first rewrite, link to PLAIN_SUMMARY, Data Access section,
  explicit disclosure that comparator responses came from free consumer interfaces
- agreement_report.md: add bootstrap 95% CIs to all kappa/ICC estimates;
  add explicit Track B divergence note (Claude κ=-0.222 vs GPT-5 κ=0.255) as
  the primary stopping rationale; caveat that floor-based PASS ≠ strong reliability
- STUDY_NARRATIVE.md: add Important Caveats section covering N=16 limitation,
  floor criterion permissiveness, mixed measurement arms, VGA reviewer disclosure,
  and calibration-to-comparator domain shift
- data/raw/README.md: placeholder documenting expected raw inputs without
  distributing confidential reviewer workbooks

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/outputs/comparator/comparator_summary_tables.xlsx
+++ b/outputs/comparator/comparator_summary_tables.xlsx
@@ -437,7 +437,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K4"/>
+  <dimension ref="A1:Y4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -468,32 +468,102 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
+          <t>validated_accuracy_ci_low</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>validated_accuracy_ci_high</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>validated_tone</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>validated_tone_ci_low</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>validated_tone_ci_high</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>validated_complementarity</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>validated_complementarity_ci_low</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>validated_complementarity_ci_high</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>validated_gilbert_urgency</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>validated_gilbert_urgency_ci_low</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>validated_gilbert_urgency_ci_high</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
         <is>
           <t>validated_discern_q7</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="R1" s="2" t="inlineStr">
+        <is>
+          <t>validated_discern_q7_ci_low</t>
+        </is>
+      </c>
+      <c r="S1" s="2" t="inlineStr">
+        <is>
+          <t>validated_discern_q7_ci_high</t>
+        </is>
+      </c>
+      <c r="T1" s="2" t="inlineStr">
         <is>
           <t>descriptive_comprehensiveness</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="U1" s="2" t="inlineStr">
+        <is>
+          <t>descriptive_comprehensiveness_ci_low</t>
+        </is>
+      </c>
+      <c r="V1" s="2" t="inlineStr">
+        <is>
+          <t>descriptive_comprehensiveness_ci_high</t>
+        </is>
+      </c>
+      <c r="W1" s="2" t="inlineStr">
         <is>
           <t>descriptive_clarity</t>
+        </is>
+      </c>
+      <c r="X1" s="2" t="inlineStr">
+        <is>
+          <t>descriptive_clarity_ci_low</t>
+        </is>
+      </c>
+      <c r="Y1" s="2" t="inlineStr">
+        <is>
+          <t>descriptive_clarity_ci_high</t>
         </is>
       </c>
     </row>
@@ -518,21 +588,63 @@
         <v>3.6875</v>
       </c>
       <c r="F2" s="3" t="n">
+        <v>3.45234375</v>
+      </c>
+      <c r="G2" s="3" t="n">
+        <v>3.939062499999999</v>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>1.65625</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="I2" s="3" t="n">
+        <v>1.46875</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>1.8125</v>
+      </c>
+      <c r="K2" s="3" t="n">
         <v>0.875</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="L2" s="3" t="n">
+        <v>0.73359375</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>0.96875</v>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>1.90625</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="O2" s="3" t="n">
+        <v>1.54609375</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>2.282812499999999</v>
+      </c>
+      <c r="Q2" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="R2" s="3" t="n">
+        <v>2.6546875</v>
+      </c>
+      <c r="S2" s="3" t="n">
+        <v>4.470312499999999</v>
+      </c>
+      <c r="T2" s="3" t="n">
         <v>4.458333333333334</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="U2" s="3" t="n">
+        <v>4.327864583333334</v>
+      </c>
+      <c r="V2" s="3" t="n">
+        <v>4.615104166666667</v>
+      </c>
+      <c r="W2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="X2" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Y2" s="3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -557,22 +669,64 @@
         <v>3.71875</v>
       </c>
       <c r="F3" s="3" t="n">
+        <v>3.54609375</v>
+      </c>
+      <c r="G3" s="3" t="n">
+        <v>3.90625</v>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>1.71875</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="I3" s="3" t="n">
+        <v>1.59375</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>1.84375</v>
+      </c>
+      <c r="K3" s="3" t="n">
         <v>0.84375</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="L3" s="3" t="n">
+        <v>0.71875</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>0.9375</v>
+      </c>
+      <c r="N3" s="3" t="n">
         <v>2.0625</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="O3" s="3" t="n">
+        <v>1.53125</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="Q3" s="3" t="n">
         <v>3.125</v>
       </c>
-      <c r="J3" s="3" t="n">
+      <c r="R3" s="3" t="n">
+        <v>2.246875</v>
+      </c>
+      <c r="S3" s="3" t="n">
+        <v>4.125</v>
+      </c>
+      <c r="T3" s="3" t="n">
         <v>4.625</v>
       </c>
-      <c r="K3" s="3" t="n">
+      <c r="U3" s="3" t="n">
+        <v>4.504427083333334</v>
+      </c>
+      <c r="V3" s="3" t="n">
+        <v>4.765885416666666</v>
+      </c>
+      <c r="W3" s="3" t="n">
         <v>4.979166666666667</v>
+      </c>
+      <c r="X3" s="3" t="n">
+        <v>4.947916666666667</v>
+      </c>
+      <c r="Y3" s="3" t="n">
+        <v>5</v>
       </c>
     </row>
     <row r="4">
@@ -596,22 +750,64 @@
         <v>3.3125</v>
       </c>
       <c r="F4" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="G4" s="3" t="n">
+        <v>3.51640625</v>
+      </c>
+      <c r="H4" s="3" t="n">
         <v>1.78125</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="I4" s="3" t="n">
+        <v>1.65625</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>1.90625</v>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>0.875</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="L4" s="3" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N4" s="3" t="n">
         <v>2.0625</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="O4" s="3" t="n">
+        <v>1.73359375</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>2.39140625</v>
+      </c>
+      <c r="Q4" s="3" t="n">
         <v>3.1875</v>
       </c>
-      <c r="J4" s="3" t="n">
+      <c r="R4" s="3" t="n">
+        <v>2.371875</v>
+      </c>
+      <c r="S4" s="3" t="n">
+        <v>3.940624999999999</v>
+      </c>
+      <c r="T4" s="3" t="n">
         <v>4.90625</v>
       </c>
-      <c r="K4" s="3" t="n">
+      <c r="U4" s="3" t="n">
+        <v>4.827864583333334</v>
+      </c>
+      <c r="V4" s="3" t="n">
+        <v>4.979166666666667</v>
+      </c>
+      <c r="W4" s="3" t="n">
         <v>4.90625</v>
+      </c>
+      <c r="X4" s="3" t="n">
+        <v>4.802083333333334</v>
+      </c>
+      <c r="Y4" s="3" t="n">
+        <v>4.989583333333334</v>
       </c>
     </row>
   </sheetData>
@@ -625,7 +821,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I6"/>
+  <dimension ref="A1:P6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -646,32 +842,67 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Original GPT-3.5 study benchmark 95% CI</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
           <t>GPT-5.5</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>GPT-5.5 95% CI</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>GPT-5.5 vs original</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
+        <is>
+          <t>GPT-5.5 vs original 95% CI</t>
+        </is>
+      </c>
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>Gemini 3.5 Flash</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash 95% CI</t>
+        </is>
+      </c>
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>Gemini 3.5 Flash vs original</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash vs original 95% CI</t>
+        </is>
+      </c>
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>Claude Sonnet 4.6</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 4.6 95% CI</t>
+        </is>
+      </c>
+      <c r="O1" s="2" t="inlineStr">
         <is>
           <t>Claude Sonnet 4.6 vs original</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 4.6 vs original 95% CI</t>
         </is>
       </c>
     </row>
@@ -689,23 +920,58 @@
       <c r="C2" s="3" t="n">
         <v>3.270833333333333</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>2.927 to 3.657</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="n">
         <v>3.6875</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>3.452 to 3.939</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>0.416666666666667</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="H2" s="3" t="inlineStr">
+        <is>
+          <t>0.010 to 0.902</t>
+        </is>
+      </c>
+      <c r="I2" s="3" t="n">
         <v>3.71875</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="J2" s="3" t="inlineStr">
+        <is>
+          <t>3.546 to 3.906</t>
+        </is>
+      </c>
+      <c r="K2" s="3" t="n">
         <v>0.447916666666667</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="L2" s="3" t="inlineStr">
+        <is>
+          <t>0.082 to 0.886</t>
+        </is>
+      </c>
+      <c r="M2" s="3" t="n">
         <v>3.3125</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="N2" s="3" t="inlineStr">
+        <is>
+          <t>3.000 to 3.516</t>
+        </is>
+      </c>
+      <c r="O2" s="3" t="n">
         <v>0.04166666666666696</v>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
+        <is>
+          <t>-0.380 to 0.459</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -722,23 +988,58 @@
       <c r="C3" s="3" t="n">
         <v>1.3125</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>1.208 to 1.438</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="n">
         <v>1.65625</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="F3" s="3" t="inlineStr">
+        <is>
+          <t>1.469 to 1.812</t>
+        </is>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>0.34375</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="H3" s="3" t="inlineStr">
+        <is>
+          <t>0.108 to 0.583</t>
+        </is>
+      </c>
+      <c r="I3" s="3" t="n">
         <v>1.71875</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="J3" s="3" t="inlineStr">
+        <is>
+          <t>1.594 to 1.844</t>
+        </is>
+      </c>
+      <c r="K3" s="3" t="n">
         <v>0.40625</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="L3" s="3" t="inlineStr">
+        <is>
+          <t>0.265 to 0.610</t>
+        </is>
+      </c>
+      <c r="M3" s="3" t="n">
         <v>1.78125</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="N3" s="3" t="inlineStr">
+        <is>
+          <t>1.656 to 1.906</t>
+        </is>
+      </c>
+      <c r="O3" s="3" t="n">
         <v>0.46875</v>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
+        <is>
+          <t>0.317 to 0.604</t>
+        </is>
       </c>
     </row>
     <row r="4">
@@ -755,23 +1056,58 @@
       <c r="C4" s="3" t="n">
         <v>0.7916666666666666</v>
       </c>
-      <c r="D4" s="3" t="n">
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>0.697 to 0.896</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="n">
         <v>0.875</v>
       </c>
-      <c r="E4" s="3" t="n">
+      <c r="F4" s="3" t="inlineStr">
+        <is>
+          <t>0.734 to 0.969</t>
+        </is>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>0.08333333333333337</v>
       </c>
-      <c r="F4" s="3" t="n">
+      <c r="H4" s="3" t="inlineStr">
+        <is>
+          <t>-0.125 to 0.251</t>
+        </is>
+      </c>
+      <c r="I4" s="3" t="n">
         <v>0.84375</v>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="J4" s="3" t="inlineStr">
+        <is>
+          <t>0.719 to 0.938</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>0.05208333333333337</v>
       </c>
-      <c r="H4" s="3" t="n">
+      <c r="L4" s="3" t="inlineStr">
+        <is>
+          <t>-0.156 to 0.208</t>
+        </is>
+      </c>
+      <c r="M4" s="3" t="n">
         <v>0.875</v>
       </c>
-      <c r="I4" s="3" t="n">
+      <c r="N4" s="3" t="inlineStr">
+        <is>
+          <t>0.750 to 1.000</t>
+        </is>
+      </c>
+      <c r="O4" s="3" t="n">
         <v>0.08333333333333337</v>
+      </c>
+      <c r="P4" s="3" t="inlineStr">
+        <is>
+          <t>-0.062 to 0.266</t>
+        </is>
       </c>
     </row>
     <row r="5">
@@ -788,23 +1124,58 @@
       <c r="C5" s="3" t="n">
         <v>2.104166666666667</v>
       </c>
-      <c r="D5" s="3" t="n">
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>1.697 to 2.490</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="n">
         <v>1.90625</v>
       </c>
-      <c r="E5" s="3" t="n">
+      <c r="F5" s="3" t="inlineStr">
+        <is>
+          <t>1.546 to 2.283</t>
+        </is>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>0.1979166666666665</v>
       </c>
-      <c r="F5" s="3" t="n">
+      <c r="H5" s="3" t="inlineStr">
+        <is>
+          <t>-0.320 to 0.761</t>
+        </is>
+      </c>
+      <c r="I5" s="3" t="n">
         <v>2.0625</v>
       </c>
-      <c r="G5" s="3" t="n">
+      <c r="J5" s="3" t="inlineStr">
+        <is>
+          <t>1.531 to 2.500</t>
+        </is>
+      </c>
+      <c r="K5" s="3" t="n">
         <v>0.04166666666666652</v>
       </c>
-      <c r="H5" s="3" t="n">
+      <c r="L5" s="3" t="inlineStr">
+        <is>
+          <t>-0.547 to 0.677</t>
+        </is>
+      </c>
+      <c r="M5" s="3" t="n">
         <v>2.0625</v>
       </c>
-      <c r="I5" s="3" t="n">
+      <c r="N5" s="3" t="inlineStr">
+        <is>
+          <t>1.734 to 2.391</t>
+        </is>
+      </c>
+      <c r="O5" s="3" t="n">
         <v>0.04166666666666652</v>
+      </c>
+      <c r="P5" s="3" t="inlineStr">
+        <is>
+          <t>-0.453 to 0.474</t>
+        </is>
       </c>
     </row>
     <row r="6">
@@ -821,23 +1192,58 @@
       <c r="C6" s="3" t="n">
         <v>3.041666666666667</v>
       </c>
-      <c r="D6" s="3" t="n">
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>2.833 to 3.230</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
         <v>3.5</v>
       </c>
-      <c r="E6" s="3" t="n">
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>2.655 to 4.470</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>0.4583333333333335</v>
       </c>
-      <c r="F6" s="3" t="n">
+      <c r="H6" s="3" t="inlineStr">
+        <is>
+          <t>-0.407 to 1.250</t>
+        </is>
+      </c>
+      <c r="I6" s="3" t="n">
         <v>3.125</v>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>2.247 to 4.125</t>
+        </is>
+      </c>
+      <c r="K6" s="3" t="n">
         <v>0.08333333333333348</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="L6" s="3" t="inlineStr">
+        <is>
+          <t>-0.826 to 1.084</t>
+        </is>
+      </c>
+      <c r="M6" s="3" t="n">
         <v>3.1875</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="N6" s="3" t="inlineStr">
+        <is>
+          <t>2.372 to 3.941</t>
+        </is>
+      </c>
+      <c r="O6" s="3" t="n">
         <v>0.1458333333333335</v>
+      </c>
+      <c r="P6" s="3" t="inlineStr">
+        <is>
+          <t>-0.604 to 0.803</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -851,7 +1257,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:Q3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -872,32 +1278,72 @@
       </c>
       <c r="D1" s="2" t="inlineStr">
         <is>
+          <t>Original GPT-3.5 study benchmark 95% CI</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
           <t>GPT-5.5</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>GPT-5.5 95% CI</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>GPT-5.5 vs original</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
+        <is>
+          <t>GPT-5.5 vs original 95% CI</t>
+        </is>
+      </c>
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>Gemini 3.5 Flash</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash 95% CI</t>
+        </is>
+      </c>
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>Gemini 3.5 Flash vs original</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
+        <is>
+          <t>Gemini 3.5 Flash vs original 95% CI</t>
+        </is>
+      </c>
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>Claude Sonnet 4.6</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="O1" s="2" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 4.6 95% CI</t>
+        </is>
+      </c>
+      <c r="P1" s="2" t="inlineStr">
         <is>
           <t>Claude Sonnet 4.6 vs original</t>
+        </is>
+      </c>
+      <c r="Q1" s="2" t="inlineStr">
+        <is>
+          <t>Claude Sonnet 4.6 vs original 95% CI</t>
         </is>
       </c>
     </row>
@@ -915,23 +1361,63 @@
       <c r="C2" s="3" t="n">
         <v>3.916666666666667</v>
       </c>
-      <c r="D2" s="3" t="n">
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>3.697 to 4.136</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Descriptive only; not validated</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="n">
         <v>4.458333333333334</v>
       </c>
-      <c r="E2" s="3" t="n">
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>4.328 to 4.615</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="n">
         <v>0.5416666666666674</v>
       </c>
-      <c r="F2" s="3" t="n">
+      <c r="I2" s="3" t="inlineStr">
+        <is>
+          <t>0.270 to 0.755</t>
+        </is>
+      </c>
+      <c r="J2" s="3" t="n">
         <v>4.625</v>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="K2" s="3" t="inlineStr">
+        <is>
+          <t>4.504 to 4.766</t>
+        </is>
+      </c>
+      <c r="L2" s="3" t="n">
         <v>0.7083333333333335</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="M2" s="3" t="inlineStr">
+        <is>
+          <t>0.462 to 0.953</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
         <v>4.90625</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="O2" s="3" t="inlineStr">
+        <is>
+          <t>4.828 to 4.979</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="n">
         <v>0.9895833333333335</v>
+      </c>
+      <c r="Q2" s="3" t="inlineStr">
+        <is>
+          <t>0.760 to 1.203</t>
+        </is>
       </c>
     </row>
     <row r="3">
@@ -948,23 +1434,63 @@
       <c r="C3" s="3" t="n">
         <v>3.770833333333333</v>
       </c>
-      <c r="D3" s="3" t="n">
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>3.604 to 3.990</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Descriptive only; not validated</t>
+        </is>
+      </c>
+      <c r="F3" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="E3" s="3" t="n">
+      <c r="G3" s="3" t="inlineStr">
+        <is>
+          <t>5.000 to 5.000</t>
+        </is>
+      </c>
+      <c r="H3" s="3" t="n">
         <v>1.229166666666667</v>
       </c>
-      <c r="F3" s="3" t="n">
+      <c r="I3" s="3" t="inlineStr">
+        <is>
+          <t>1.020 to 1.417</t>
+        </is>
+      </c>
+      <c r="J3" s="3" t="n">
         <v>4.979166666666667</v>
       </c>
-      <c r="G3" s="3" t="n">
+      <c r="K3" s="3" t="inlineStr">
+        <is>
+          <t>4.948 to 5.000</t>
+        </is>
+      </c>
+      <c r="L3" s="3" t="n">
         <v>1.208333333333333</v>
       </c>
-      <c r="H3" s="3" t="n">
+      <c r="M3" s="3" t="inlineStr">
+        <is>
+          <t>1.026 to 1.417</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="n">
         <v>4.90625</v>
       </c>
-      <c r="I3" s="3" t="n">
+      <c r="O3" s="3" t="inlineStr">
+        <is>
+          <t>4.802 to 4.990</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="n">
         <v>1.135416666666667</v>
+      </c>
+      <c r="Q3" s="3" t="inlineStr">
+        <is>
+          <t>0.911 to 1.302</t>
+        </is>
       </c>
     </row>
   </sheetData>
@@ -1064,7 +1590,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:G8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1090,6 +1616,16 @@
       </c>
       <c r="E1" s="2" t="inlineStr">
         <is>
+          <t>original_mean_ci_low</t>
+        </is>
+      </c>
+      <c r="F1" s="2" t="inlineStr">
+        <is>
+          <t>original_mean_ci_high</t>
+        </is>
+      </c>
+      <c r="G1" s="2" t="inlineStr">
+        <is>
           <t>response_count</t>
         </is>
       </c>
@@ -1114,6 +1650,12 @@
         <v>3.270833333333333</v>
       </c>
       <c r="E2" s="3" t="n">
+        <v>2.9265625</v>
+      </c>
+      <c r="F2" s="3" t="n">
+        <v>3.656770833333333</v>
+      </c>
+      <c r="G2" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1137,6 +1679,12 @@
         <v>1.3125</v>
       </c>
       <c r="E3" s="3" t="n">
+        <v>1.208333333333333</v>
+      </c>
+      <c r="F3" s="3" t="n">
+        <v>1.4375</v>
+      </c>
+      <c r="G3" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1160,6 +1708,12 @@
         <v>0.7916666666666666</v>
       </c>
       <c r="E4" s="3" t="n">
+        <v>0.6973958333333333</v>
+      </c>
+      <c r="F4" s="3" t="n">
+        <v>0.8958333333333333</v>
+      </c>
+      <c r="G4" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1183,6 +1737,12 @@
         <v>2.104166666666667</v>
       </c>
       <c r="E5" s="3" t="n">
+        <v>1.697395833333333</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>2.490104166666667</v>
+      </c>
+      <c r="G5" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1206,6 +1766,12 @@
         <v>3.041666666666667</v>
       </c>
       <c r="E6" s="3" t="n">
+        <v>2.833333333333333</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>3.230208333333333</v>
+      </c>
+      <c r="G6" s="3" t="n">
         <v>8</v>
       </c>
     </row>
@@ -1229,6 +1795,12 @@
         <v>3.916666666666667</v>
       </c>
       <c r="E7" s="3" t="n">
+        <v>3.697395833333333</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>4.1359375</v>
+      </c>
+      <c r="G7" s="3" t="n">
         <v>16</v>
       </c>
     </row>
@@ -1252,6 +1824,12 @@
         <v>3.770833333333333</v>
       </c>
       <c r="E8" s="3" t="n">
+        <v>3.604166666666667</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>3.990104166666666</v>
+      </c>
+      <c r="G8" s="3" t="n">
         <v>16</v>
       </c>
     </row>

</xml_diff>